<commit_message>
add capta sur mail
</commit_message>
<xml_diff>
--- a/Tableau_de_synthese.xlsx
+++ b/Tableau_de_synthese.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\BTS_SIO_portfolio\BTS_SIO_portofolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0172B0F6-E2BA-4065-AFE9-365D588DDCAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F33E491-147D-464F-8308-1D20789ECE50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="45">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -182,6 +182,18 @@
   </si>
   <si>
     <t>​☒ SISR</t>
+  </si>
+  <si>
+    <t>utilisation d'un Linux sans GUI (chez moi)</t>
+  </si>
+  <si>
+    <t>script automatisation de la configuration Windows Server (création d’OU, création d'utilisateur, intégration des utilisateurs dans des UO)</t>
+  </si>
+  <si>
+    <t>Script d'automatisation (fichier unattend) d'installation de Windows 11</t>
+  </si>
+  <si>
+    <t>Installation VM  Linux Arch</t>
   </si>
 </sst>
 </file>
@@ -718,9 +730,48 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -743,45 +794,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1103,56 +1115,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="22"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="29" t="s">
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="24"/>
-      <c r="H3" s="30"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="43"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="28"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="12" t="s">
         <v>4</v>
       </c>
@@ -1164,22 +1176,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="35"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1202,8 +1214,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="32"/>
-      <c r="B7" s="40"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="20" t="s">
         <v>14</v>
       </c>
@@ -1259,16 +1271,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="35"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="27"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1847,16 +1859,16 @@
       <c r="AQ19"/>
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="38"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="30"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1894,7 +1906,9 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
+      <c r="A21" s="9" t="s">
+        <v>44</v>
+      </c>
       <c r="B21" s="8"/>
       <c r="C21" s="15"/>
       <c r="D21" s="15"/>
@@ -2209,16 +2223,16 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A28" s="36" t="s">
+      <c r="A28" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="37"/>
-      <c r="C28" s="37"/>
-      <c r="D28" s="37"/>
-      <c r="E28" s="37"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="37"/>
-      <c r="H28" s="38"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="30"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2350,7 +2364,9 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="9"/>
+      <c r="A31" s="9" t="s">
+        <v>41</v>
+      </c>
       <c r="B31" s="8"/>
       <c r="C31" s="15"/>
       <c r="D31" s="15"/>
@@ -2395,7 +2411,9 @@
       <c r="AQ31"/>
     </row>
     <row r="32" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="9"/>
+      <c r="A32" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="B32" s="8"/>
       <c r="C32" s="15"/>
       <c r="D32" s="15"/>
@@ -2440,7 +2458,9 @@
       <c r="AQ32"/>
     </row>
     <row r="33" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="9"/>
+      <c r="A33" s="9" t="s">
+        <v>43</v>
+      </c>
       <c r="B33" s="8"/>
       <c r="C33" s="15"/>
       <c r="D33" s="15"/>
@@ -2667,6 +2687,11 @@
     <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2674,11 +2699,6 @@
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2689,15 +2709,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BA30588C50A37641B2E228799579EC11" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="05fd44df0ba32ce0d87b46c7cf206d9a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c1552a64-ca45-4253-b609-1c6027926d23" xmlns:ns3="8f0af72c-24f0-4a1d-bef0-182580005356" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6166865f7e1a0e28c47b1a017d6c1fe4" ns2:_="" ns3:_="">
     <xsd:import namespace="c1552a64-ca45-4253-b609-1c6027926d23"/>
@@ -2898,6 +2909,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2910,14 +2930,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A16B3B8-77F0-4ABA-B408-0F1A4EB64D06}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C022D49A-AE61-4E7C-A6F4-B87FD5986203}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2936,6 +2948,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A16B3B8-77F0-4ABA-B408-0F1A4EB64D06}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78FDA2C8-9146-4C05-BFE6-881AEDABADDC}">
   <ds:schemaRefs>

</xml_diff>